<commit_message>
fix: unit is person weeks. Assume absence has uniform distribution
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/examples/input_example.xlsx
+++ b/data/examples/input_example.xlsx
@@ -1,34 +1,103 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
   <workbookPr/>
-  <workbookProtection/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/irina.migallon/dev/cli/planzen/data/examples/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68070D5F-8FE2-1048-B830-A96815D64B20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Plan" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Plan" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="20">
+  <si>
+    <t>Epics</t>
+  </si>
+  <si>
+    <t>Estimation</t>
+  </si>
+  <si>
+    <t>Budget Bucket</t>
+  </si>
+  <si>
+    <t>Priority</t>
+  </si>
+  <si>
+    <t>Milestone</t>
+  </si>
+  <si>
+    <t>Auth &amp; Identity Management</t>
+  </si>
+  <si>
+    <t>Platform</t>
+  </si>
+  <si>
+    <t>Q1</t>
+  </si>
+  <si>
+    <t>Real-time Analytics</t>
+  </si>
+  <si>
+    <t>Analytics</t>
+  </si>
+  <si>
+    <t>Q2</t>
+  </si>
+  <si>
+    <t>Mobile App Redesign</t>
+  </si>
+  <si>
+    <t>Product</t>
+  </si>
+  <si>
+    <t>API Gateway Optimization</t>
+  </si>
+  <si>
+    <t>Q3</t>
+  </si>
+  <si>
+    <t>Data Quality Framework</t>
+  </si>
+  <si>
+    <t>Engineers capacity</t>
+  </si>
+  <si>
+    <t>Managers capacity</t>
+  </si>
+  <si>
+    <t>Engineers absence</t>
+  </si>
+  <si>
+    <t>Managers absence</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -47,80 +116,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -408,157 +418,151 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:E11"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Epics</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Estimation</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Budget Bucket</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Priority</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Milestone</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Auth &amp; Identity Management</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2">
         <v>80</v>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Platform</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
+      <c r="C2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2">
         <v>0</v>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Q1</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Real-time Analytics</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
+      <c r="E2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3">
         <v>120</v>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Analytics</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
+      <c r="C3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3">
         <v>0</v>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Q2</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Mobile App Redesign</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
+      <c r="E3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4">
         <v>100</v>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
+      <c r="C4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4">
         <v>1</v>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Q2</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>API Gateway Optimization</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
+      <c r="E4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5">
         <v>60</v>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Platform</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
+      <c r="C5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D5">
         <v>1</v>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Q3</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Data Quality Framework</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
+      <c r="E5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6">
         <v>90</v>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Analytics</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
+      <c r="C6" t="s">
+        <v>9</v>
+      </c>
+      <c r="D6">
         <v>2</v>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Q3</t>
-        </is>
+      <c r="E6" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>17</v>
+      </c>
+      <c r="B9">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>18</v>
+      </c>
+      <c r="B10">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>19</v>
+      </c>
+      <c r="B11">
+        <v>0.5</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{7191b2d3-7d38-48ed-b3a4-7a9f420ca5cd}" enabled="1" method="Standard" siteId="{374f8026-7b54-4a3a-b87d-328fa26ec10d}" contentBits="0" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>

<commit_message>
feat: move team config to Excel and auto-derive timestamped output paths
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/examples/input_example.xlsx
+++ b/data/examples/input_example.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -456,110 +456,56 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Auth &amp; Identity Management</t>
+          <t>Engineer Bruto Capacity</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>80</v>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Platform</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Feature</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>https://jira.example.com/AUTH-1</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Q1</t>
-        </is>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Real-time Analytics</t>
+          <t>Management Bruto Capacity</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>120</v>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Analytics</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Feature</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>https://jira.example.com/ANA-1</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Q2</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Mobile App Redesign</t>
+          <t>Engineer Absence (days)</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>100</v>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Improvement</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>https://jira.example.com/MOB-1</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Q2</t>
-        </is>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>API Gateway Optimization</t>
+          <t>Auth &amp; Identity Management</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -568,51 +514,150 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Improvement</t>
+          <t>Feature</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://jira.example.com/API-1</t>
+          <t>https://jira.example.com/AUTH-1</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Q3</t>
+          <t>Q1</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>Real-time Analytics</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>120</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Analytics</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>https://jira.example.com/ANA-1</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Mobile App Redesign</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>100</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Improvement</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>https://jira.example.com/MOB-1</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>API Gateway Optimization</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>60</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Improvement</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>https://jira.example.com/API-1</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>Data Quality Framework</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="B9" t="n">
         <v>90</v>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>Analytics</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>Feature</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>https://jira.example.com/DQ-1</t>
         </is>
       </c>
-      <c r="F6" t="n">
+      <c r="F9" t="n">
         <v>2</v>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>Q3</t>
         </is>

</xml_diff>

<commit_message>
feat: validate input, fuzzy config label matching, Type optional
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/examples/input_example.xlsx
+++ b/data/examples/input_example.xlsx
@@ -471,7 +471,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Management Bruto Capacity</t>
+          <t>Manager Bruto Capacity</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -501,15 +501,15 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Auth &amp; Identity Management</t>
+          <t>Alpha Search</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>80</v>
+        <v>8</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Platform</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -519,44 +519,44 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://jira.example.com/AUTH-1</t>
+          <t>http://jira/1</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Q1</t>
+          <t>Q2</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Real-time Analytics</t>
+          <t>Beta Platform</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>120</v>
+        <v>12</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Analytics</t>
+          <t>Platform</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Feature</t>
+          <t>Tech Debt</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://jira.example.com/ANA-1</t>
+          <t>http://jira/2</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -567,29 +567,29 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Mobile App Redesign</t>
+          <t>Gamma Onboarding</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>100</v>
+        <v>5</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>Growth</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Improvement</t>
+          <t>Feature</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://jira.example.com/MOB-1</t>
+          <t>http://jira/3</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -600,11 +600,11 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>API Gateway Optimization</t>
+          <t>Delta Infra</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>60</v>
+        <v>7</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -618,48 +618,48 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://jira.example.com/API-1</t>
+          <t>http://jira/4</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Q3</t>
+          <t>Q2</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Data Quality Framework</t>
+          <t>Epsilon Compliance</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>90</v>
+        <v>3</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Analytics</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Feature</t>
+          <t>Compliance</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://jira.example.com/DQ-1</t>
+          <t>http://jira/5</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Q3</t>
+          <t>Q2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: allocation modes (Sprint/Uniform/Gaps) and auto-overflow
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>

fix: auto-overflow was not complete
</commit_message>
<xml_diff>
--- a/data/examples/input_example.xlsx
+++ b/data/examples/input_example.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -452,6 +452,11 @@
           <t>Milestone</t>
         </is>
       </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Allocation Mode</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -462,11 +467,6 @@
       <c r="B2" t="n">
         <v>5</v>
       </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -477,11 +477,6 @@
       <c r="B3" t="n">
         <v>2</v>
       </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -492,11 +487,6 @@
       <c r="B4" t="n">
         <v>10</v>
       </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -563,6 +553,11 @@
           <t>Q2</t>
         </is>
       </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Sprint</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -596,6 +591,11 @@
           <t>Q2</t>
         </is>
       </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Uniform</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -627,6 +627,11 @@
       <c r="G8" t="inlineStr">
         <is>
           <t>Q2</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Gaps allowed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: config rows in Budget Bucket, robust column loading, empty estimation defaults to 0
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/examples/input_example.xlsx
+++ b/data/examples/input_example.xlsx
@@ -459,34 +459,52 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Engineer Bruto Capacity</t>
-        </is>
-      </c>
+      <c r="A2" t="inlineStr"/>
       <c r="B2" t="n">
         <v>5</v>
       </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Engineer Capacity (Bruto)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Manager Bruto Capacity</t>
-        </is>
-      </c>
+      <c r="A3" t="inlineStr"/>
       <c r="B3" t="n">
         <v>2</v>
       </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Management Capacity (Bruto)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Engineer Absence (days)</t>
-        </is>
-      </c>
+      <c r="A4" t="inlineStr"/>
       <c r="B4" t="n">
         <v>10</v>
       </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Engineer Absence</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -520,6 +538,7 @@
           <t>Q2</t>
         </is>
       </c>
+      <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -631,7 +650,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Gaps allowed</t>
+          <t>Gaps</t>
         </is>
       </c>
     </row>
@@ -667,6 +686,7 @@
           <t>Q2</t>
         </is>
       </c>
+      <c r="H9" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>